<commit_message>
vault backup: 2026-10-17 10:12:11
</commit_message>
<xml_diff>
--- a/vault/02_주요진행상황/업계섭외현황.xlsx
+++ b/vault/02_주요진행상황/업계섭외현황.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\뉴프로젝트\2026dgs\vault\02_주요진행상황\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C64C95D6-847C-4699-87B6-5E92E578327E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D4DA202-2D97-4E5F-8015-1D59CC32D02F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28305" yWindow="-450" windowWidth="16860" windowHeight="14970" xr2:uid="{01041B61-266B-4521-86E9-FF95823D999B}"/>
+    <workbookView xWindow="-27240" yWindow="-255" windowWidth="16860" windowHeight="14970" xr2:uid="{01041B61-266B-4521-86E9-FF95823D999B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="97">
   <si>
     <t>일련
 번호</t>
@@ -415,6 +415,10 @@
   <si>
     <t>참가의향 메일발송</t>
     <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>참석 회신</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1365,7 +1369,9 @@
       <c r="H13" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="I13" s="2"/>
+      <c r="I13" s="2" t="s">
+        <v>93</v>
+      </c>
       <c r="J13" s="2"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
@@ -1393,7 +1399,9 @@
       <c r="H14" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="I14" s="2"/>
+      <c r="I14" s="2" t="s">
+        <v>96</v>
+      </c>
       <c r="J14" s="2"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
@@ -1509,7 +1517,9 @@
       <c r="H18" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="I18" s="3"/>
+      <c r="I18" s="3" t="s">
+        <v>96</v>
+      </c>
       <c r="J18" s="3"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">

</xml_diff>